<commit_message>
chore: snapshot current warehouse source
</commit_message>
<xml_diff>
--- a/docs/mau_nhap_nha_kho.xlsx
+++ b/docs/mau_nhap_nha_kho.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Nha_kho" sheetId="1" r:id="rId1"/>
+    <sheet name="Danh_muc" sheetId="2" r:id="rId2" state="hidden"/>
   </sheets>
 </workbook>
 </file>
@@ -397,244 +398,419 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:AA3"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="23.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="17.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
+    <col min="22" max="22" width="26.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>cap_1</v>
+      </c>
+      <c r="B1" t="str">
+        <v>cap_2</v>
+      </c>
+      <c r="C1" t="str">
+        <v>cap_3</v>
+      </c>
+      <c r="D1" t="str">
+        <v>cap_4</v>
+      </c>
+      <c r="E1" t="str">
+        <v>cap_5</v>
+      </c>
+      <c r="F1" t="str">
+        <v>cap_6</v>
+      </c>
+      <c r="G1" t="str">
         <v>name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="H1" t="str">
         <v>address</v>
       </c>
-      <c r="C1" t="str">
+      <c r="I1" t="str">
         <v>warehouse_category</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J1" t="str">
         <v>quantity</v>
       </c>
-      <c r="E1" t="str">
+      <c r="K1" t="str">
         <v>land_area</v>
       </c>
-      <c r="F1" t="str">
+      <c r="L1" t="str">
         <v>warehouse_area</v>
       </c>
-      <c r="G1" t="str">
+      <c r="M1" t="str">
         <v>warehouse_land_area</v>
       </c>
-      <c r="H1" t="str">
+      <c r="N1" t="str">
         <v>year_built</v>
       </c>
-      <c r="I1" t="str">
+      <c r="O1" t="str">
         <v>year_renovated</v>
       </c>
-      <c r="J1" t="str">
+      <c r="P1" t="str">
         <v>storage_capacity</v>
       </c>
-      <c r="K1" t="str">
+      <c r="Q1" t="str">
         <v>current_stock</v>
       </c>
-      <c r="L1" t="str">
+      <c r="R1" t="str">
         <v>quality_grade_23_area</v>
       </c>
-      <c r="M1" t="str">
+      <c r="S1" t="str">
         <v>quality_grade_4_area</v>
       </c>
-      <c r="N1" t="str">
+      <c r="T1" t="str">
         <v>temp_house_area</v>
       </c>
-      <c r="O1" t="str">
+      <c r="U1" t="str">
         <v>lightning_grade_area</v>
       </c>
-      <c r="P1" t="str">
+      <c r="V1" t="str">
         <v>lightning_existing_count</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="W1" t="str">
         <v>fire_need</v>
       </c>
-      <c r="R1" t="str">
+      <c r="X1" t="str">
         <v>fire_existing</v>
       </c>
-      <c r="S1" t="str">
+      <c r="Y1" t="str">
         <v>notes</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>unit_type</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>unit_id</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kho VKTB Tổng hợp 01</v>
+        <v>Tổng cục</v>
       </c>
       <c r="B2" t="str">
-        <v>Phường Bạch Đằng, TP Hải Phòng</v>
+        <v>Vùng 1</v>
       </c>
       <c r="C2" t="str">
+        <v>Lữ 7</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Phòng kỹ thuật</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Nhà kho 7</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Kho K1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Kho K1</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>chien_thuat</v>
       </c>
-      <c r="D2">
+      <c r="J2">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>500</v>
-      </c>
-      <c r="F2">
-        <v>350</v>
-      </c>
-      <c r="G2">
-        <v>450</v>
-      </c>
-      <c r="H2">
-        <v>2015</v>
-      </c>
-      <c r="I2">
-        <v>2023</v>
-      </c>
-      <c r="J2">
-        <v>80</v>
-      </c>
       <c r="K2">
-        <v>55</v>
+        <v>600</v>
       </c>
       <c r="L2">
-        <v>200</v>
+        <v>420</v>
       </c>
       <c r="M2">
+        <v>520</v>
+      </c>
+      <c r="N2">
+        <v>2018</v>
+      </c>
+      <c r="O2">
+        <v>2024</v>
+      </c>
+      <c r="P2">
         <v>100</v>
       </c>
-      <c r="N2">
-        <v>50</v>
-      </c>
-      <c r="O2">
-        <v>350</v>
-      </c>
-      <c r="P2">
+      <c r="Q2">
+        <v>60</v>
+      </c>
+      <c r="R2">
+        <v>300</v>
+      </c>
+      <c r="S2">
+        <v>100</v>
+      </c>
+      <c r="T2">
+        <v>20</v>
+      </c>
+      <c r="U2">
+        <v>420</v>
+      </c>
+      <c r="V2">
         <v>2</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="W2" t="str">
         <v>Cần thiết</v>
       </c>
-      <c r="R2" t="str">
+      <c r="X2" t="str">
         <v>Có</v>
       </c>
-      <c r="S2" t="str">
-        <v>Dữ liệu mẫu — kho chiến thuật vùng 1</v>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v>warehouse</v>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Kho Xăng dầu K02</v>
+        <v>Tổng cục</v>
       </c>
       <c r="B3" t="str">
-        <v>Phường Hà Tu, TP Hạ Long, Quảng Ninh</v>
+        <v>Vùng 1</v>
       </c>
       <c r="C3" t="str">
+        <v>Lữ 7</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Phòng kỹ thuật</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>Nhà kho 7</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Nhà kho 7</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>chien_dich</v>
       </c>
-      <c r="D3">
+      <c r="J3">
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="K3">
         <v>1200</v>
       </c>
-      <c r="F3">
-        <v>900</v>
-      </c>
-      <c r="G3">
-        <v>1100</v>
-      </c>
-      <c r="H3">
-        <v>2010</v>
-      </c>
-      <c r="I3">
-        <v>2024</v>
-      </c>
-      <c r="J3">
+      <c r="L3">
+        <v>850</v>
+      </c>
+      <c r="M3">
+        <v>1000</v>
+      </c>
+      <c r="N3">
+        <v>2016</v>
+      </c>
+      <c r="O3">
+        <v>2023</v>
+      </c>
+      <c r="P3">
         <v>250</v>
       </c>
-      <c r="K3">
+      <c r="Q3">
         <v>180</v>
       </c>
-      <c r="L3">
-        <v>500</v>
-      </c>
-      <c r="M3">
-        <v>300</v>
-      </c>
-      <c r="N3">
-        <v>100</v>
-      </c>
-      <c r="O3">
-        <v>900</v>
-      </c>
-      <c r="P3">
+      <c r="R3">
+        <v>650</v>
+      </c>
+      <c r="S3">
+        <v>150</v>
+      </c>
+      <c r="T3">
+        <v>50</v>
+      </c>
+      <c r="U3">
+        <v>850</v>
+      </c>
+      <c r="V3">
         <v>4</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="W3" t="str">
         <v>Cần thiết</v>
       </c>
-      <c r="R3" t="str">
+      <c r="X3" t="str">
         <v>Có</v>
       </c>
-      <c r="S3" t="str">
-        <v>Kho chiến dịch — xăng dầu</v>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v>warehouse</v>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>cap_1</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tổng cục</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>cap_2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Vùng 1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Vùng 2</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Vùng 3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>cap_3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lữ 7</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Lữ 8</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Lữ 9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Kho Lương thực K03</v>
+        <v>cap_4</v>
       </c>
       <c r="B4" t="str">
-        <v>Xã Hải An, Huyện Thủy Nguyên, Hải Phòng</v>
+        <v>Phòng kỹ thuật</v>
       </c>
       <c r="C4" t="str">
+        <v>Phòng hậu cần</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ban kho</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>cap_5</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Nhà kho 7</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nhà kho 8</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Kho trung tâm</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>cap_6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Kho K1</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Kho K2</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kho K3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>warehouse_category</v>
+      </c>
+      <c r="B7" t="str">
         <v>chien_thuat</v>
       </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>800</v>
-      </c>
-      <c r="F4">
-        <v>600</v>
-      </c>
-      <c r="G4">
-        <v>750</v>
-      </c>
-      <c r="H4">
-        <v>2018</v>
-      </c>
-      <c r="J4">
-        <v>120</v>
-      </c>
-      <c r="K4">
-        <v>90</v>
-      </c>
-      <c r="L4">
-        <v>400</v>
-      </c>
-      <c r="M4">
-        <v>150</v>
-      </c>
-      <c r="N4">
-        <v>50</v>
-      </c>
-      <c r="O4">
-        <v>600</v>
-      </c>
-      <c r="P4">
-        <v>3</v>
-      </c>
-      <c r="Q4" t="str">
+      <c r="C7" t="str">
+        <v>chien_dich</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>fire_need</v>
+      </c>
+      <c r="B8" t="str">
         <v>Cần thiết</v>
       </c>
-      <c r="R4" t="str">
+      <c r="C8" t="str">
+        <v>Không cần</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>fire_existing</v>
+      </c>
+      <c r="B9" t="str">
         <v>Có</v>
       </c>
-      <c r="S4" t="str">
-        <v>Kho lương thực dự trữ</v>
+      <c r="C9" t="str">
+        <v>Không</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>unit_type</v>
+      </c>
+      <c r="B10" t="str">
+        <v>warehouse</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>